<commit_message>
agregado datos de prueba
</commit_message>
<xml_diff>
--- a/autos_prod.xlsx
+++ b/autos_prod.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11109"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Joaco\Desktop\granos_downloader\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/juan/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{284113AC-7D56-4F9C-8621-24C0934CE453}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9A239F2F-76B2-6740-B27B-A3800CC35049}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3030" yWindow="3030" windowWidth="21600" windowHeight="11385" xr2:uid="{86125D5C-7730-A64B-9963-5E39821F9F28}"/>
+    <workbookView xWindow="26780" yWindow="15600" windowWidth="25640" windowHeight="14440" xr2:uid="{86125D5C-7730-A64B-9963-5E39821F9F28}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
   <numFmts count="3">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_-* #,##0.0_-;\-* #,##0.0_-;_-* &quot;-&quot;?_-;_-@_-"/>
-    <numFmt numFmtId="165" formatCode="_-* #,##0.0_-;\-* #,##0.0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="166" formatCode="_-* #,##0.0_-;\-* #,##0.0_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -89,7 +89,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Millares" xfId="1" builtinId="3"/>
@@ -426,9 +426,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E6D3223-9B34-7749-9750-BC6E8F2692D1}">
   <dimension ref="A1:C388"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="1">
         <v>34335</v>
       </c>
@@ -439,7 +439,7 @@
         <v>54184.919853681902</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
         <v>34366</v>
       </c>
@@ -450,7 +450,7 @@
         <v>11377.410415660001</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
         <v>34394</v>
       </c>
@@ -461,7 +461,7 @@
         <v>27975.131324678299</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
         <v>34425</v>
       </c>
@@ -472,7 +472,7 @@
         <v>34619.232720471198</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
         <v>34455</v>
       </c>
@@ -483,7 +483,7 @@
         <v>29650.927593224598</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
         <v>34486</v>
       </c>
@@ -494,7 +494,7 @@
         <v>31585.568568543698</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
         <v>34516</v>
       </c>
@@ -505,7 +505,7 @@
         <v>32738.744906158299</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
         <v>34547</v>
       </c>
@@ -516,7 +516,7 @@
         <v>34574.880033895803</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
         <v>34578</v>
       </c>
@@ -527,7 +527,7 @@
         <v>35853.527564119497</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
         <v>34608</v>
       </c>
@@ -538,7 +538,7 @@
         <v>34197.938022183698</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
         <v>34639</v>
       </c>
@@ -549,7 +549,7 @@
         <v>33917.7733169766</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
         <v>34669</v>
       </c>
@@ -560,7 +560,7 @@
         <v>32998.406600299502</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
         <v>34700</v>
       </c>
@@ -571,7 +571,7 @@
         <v>27377.563106936301</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
         <v>34731</v>
       </c>
@@ -582,7 +582,7 @@
         <v>35724.345782012802</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
         <v>34759</v>
       </c>
@@ -593,7 +593,7 @@
         <v>30041.463004886598</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" s="1">
         <v>34790</v>
       </c>
@@ -604,7 +604,7 @@
         <v>25523.124279007199</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" s="1">
         <v>34820</v>
       </c>
@@ -615,7 +615,7 @@
         <v>25067.731543215599</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" s="1">
         <v>34851</v>
       </c>
@@ -626,7 +626,7 @@
         <v>18988.896923801702</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" s="1">
         <v>34881</v>
       </c>
@@ -637,7 +637,7 @@
         <v>19800.092567661399</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" s="1">
         <v>34912</v>
       </c>
@@ -648,7 +648,7 @@
         <v>16745.827759619799</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" s="1">
         <v>34943</v>
       </c>
@@ -659,7 +659,7 @@
         <v>16960.4863945785</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" s="1">
         <v>34973</v>
       </c>
@@ -670,7 +670,7 @@
         <v>18049.109994197301</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" s="1">
         <v>35004</v>
       </c>
@@ -681,7 +681,7 @@
         <v>18684.519614650999</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" s="1">
         <v>35034</v>
       </c>
@@ -692,7 +692,7 @@
         <v>21960.583303994099</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" s="1">
         <v>35065</v>
       </c>
@@ -703,7 +703,7 @@
         <v>21608.389458003501</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" s="1">
         <v>35096</v>
       </c>
@@ -714,7 +714,7 @@
         <v>25070.950698786401</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" s="1">
         <v>35125</v>
       </c>
@@ -725,7 +725,7 @@
         <v>23221.784570876898</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" s="1">
         <v>35156</v>
       </c>
@@ -736,7 +736,7 @@
         <v>24418.130845783598</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A29" s="1">
         <v>35186</v>
       </c>
@@ -747,7 +747,7 @@
         <v>24085.058829388101</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A30" s="1">
         <v>35217</v>
       </c>
@@ -758,7 +758,7 @@
         <v>26143.3913308585</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A31" s="1">
         <v>35247</v>
       </c>
@@ -769,7 +769,7 @@
         <v>25408.346574961499</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A32" s="1">
         <v>35278</v>
       </c>
@@ -780,7 +780,7 @@
         <v>26721.123785518401</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A33" s="1">
         <v>35309</v>
       </c>
@@ -791,7 +791,7 @@
         <v>23844.175430935102</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A34" s="1">
         <v>35339</v>
       </c>
@@ -802,7 +802,7 @@
         <v>26318.523451090001</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A35" s="1">
         <v>35370</v>
       </c>
@@ -813,7 +813,7 @@
         <v>28553.208084188602</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A36" s="1">
         <v>35400</v>
       </c>
@@ -824,7 +824,7 @@
         <v>27780.878732873</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A37" s="1">
         <v>35431</v>
       </c>
@@ -835,7 +835,7 @@
         <v>30316.584082667501</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A38" s="1">
         <v>35462</v>
       </c>
@@ -846,7 +846,7 @@
         <v>29783.183503449902</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A39" s="1">
         <v>35490</v>
       </c>
@@ -857,7 +857,7 @@
         <v>31266.826704029001</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A40" s="1">
         <v>35521</v>
       </c>
@@ -868,7 +868,7 @@
         <v>33424.059481946402</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A41" s="1">
         <v>35551</v>
       </c>
@@ -879,7 +879,7 @@
         <v>34511.587308119299</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A42" s="1">
         <v>35582</v>
       </c>
@@ -890,7 +890,7 @@
         <v>35496.090419817403</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A43" s="1">
         <v>35612</v>
       </c>
@@ -901,7 +901,7 @@
         <v>37058.324771455802</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A44" s="1">
         <v>35643</v>
       </c>
@@ -912,7 +912,7 @@
         <v>37552.537486997899</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A45" s="1">
         <v>35674</v>
       </c>
@@ -923,7 +923,7 @@
         <v>39091.2937447718</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A46" s="1">
         <v>35704</v>
       </c>
@@ -934,7 +934,7 @@
         <v>46856.699261907001</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A47" s="1">
         <v>35735</v>
       </c>
@@ -945,7 +945,7 @@
         <v>42623.626518107798</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A48" s="1">
         <v>35765</v>
       </c>
@@ -956,7 +956,7 @@
         <v>26341.308605894701</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A49" s="1">
         <v>35796</v>
       </c>
@@ -967,7 +967,7 @@
         <v>34616.6059526479</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A50" s="1">
         <v>35827</v>
       </c>
@@ -978,7 +978,7 @@
         <v>37689.402208084502</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A51" s="1">
         <v>35855</v>
       </c>
@@ -989,7 +989,7 @@
         <v>39230.018131008299</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A52" s="1">
         <v>35886</v>
       </c>
@@ -1000,7 +1000,7 @@
         <v>40105.368967091599</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A53" s="1">
         <v>35916</v>
       </c>
@@ -1011,7 +1011,7 @@
         <v>39621.004503797798</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A54" s="1">
         <v>35947</v>
       </c>
@@ -1022,7 +1022,7 @@
         <v>41146.906094480699</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A55" s="1">
         <v>35977</v>
       </c>
@@ -1033,7 +1033,7 @@
         <v>39163.537041550997</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A56" s="1">
         <v>36008</v>
       </c>
@@ -1044,7 +1044,7 @@
         <v>44666.293578942103</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A57" s="1">
         <v>36039</v>
       </c>
@@ -1055,7 +1055,7 @@
         <v>39507.388652230497</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A58" s="1">
         <v>36069</v>
       </c>
@@ -1066,7 +1066,7 @@
         <v>34305.091007386203</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A59" s="1">
         <v>36100</v>
       </c>
@@ -1077,7 +1077,7 @@
         <v>28983.738455854102</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A60" s="1">
         <v>36130</v>
       </c>
@@ -1088,7 +1088,7 @@
         <v>15343.033591760601</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A61" s="1">
         <v>36161</v>
       </c>
@@ -1099,7 +1099,7 @@
         <v>27624.387690503401</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A62" s="1">
         <v>36192</v>
       </c>
@@ -1110,7 +1110,7 @@
         <v>20762.024560814101</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A63" s="1">
         <v>36220</v>
       </c>
@@ -1121,7 +1121,7 @@
         <v>18046.1306319453</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A64" s="1">
         <v>36251</v>
       </c>
@@ -1132,7 +1132,7 @@
         <v>18642.089562739999</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A65" s="1">
         <v>36281</v>
       </c>
@@ -1143,7 +1143,7 @@
         <v>21853.531798893298</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A66" s="1">
         <v>36312</v>
       </c>
@@ -1154,7 +1154,7 @@
         <v>21591.239228119299</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A67" s="1">
         <v>36342</v>
       </c>
@@ -1165,7 +1165,7 @@
         <v>22443.148876883999</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A68" s="1">
         <v>36373</v>
       </c>
@@ -1176,7 +1176,7 @@
         <v>25381.910034239801</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A69" s="1">
         <v>36404</v>
       </c>
@@ -1187,7 +1187,7 @@
         <v>24281.778176861299</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A70" s="1">
         <v>36434</v>
       </c>
@@ -1198,7 +1198,7 @@
         <v>28724.3541712265</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A71" s="1">
         <v>36465</v>
       </c>
@@ -1209,7 +1209,7 @@
         <v>29348.663139907901</v>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A72" s="1">
         <v>36495</v>
       </c>
@@ -1220,7 +1220,7 @@
         <v>32374.5826176501</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A73" s="1">
         <v>36526</v>
       </c>
@@ -1231,7 +1231,7 @@
         <v>38018.561463152502</v>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A74" s="1">
         <v>36557</v>
       </c>
@@ -1242,7 +1242,7 @@
         <v>26947.517213094499</v>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A75" s="1">
         <v>36586</v>
       </c>
@@ -1253,7 +1253,7 @@
         <v>30664.298202580299</v>
       </c>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A76" s="1">
         <v>36617</v>
       </c>
@@ -1264,7 +1264,7 @@
         <v>28588.474456038199</v>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A77" s="1">
         <v>36647</v>
       </c>
@@ -1275,7 +1275,7 @@
         <v>25318.404791981498</v>
       </c>
     </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A78" s="1">
         <v>36678</v>
       </c>
@@ -1286,7 +1286,7 @@
         <v>24503.403937364699</v>
       </c>
     </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A79" s="1">
         <v>36708</v>
       </c>
@@ -1297,7 +1297,7 @@
         <v>26309.1755642186</v>
       </c>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A80" s="1">
         <v>36739</v>
       </c>
@@ -1308,7 +1308,7 @@
         <v>24617.533326077701</v>
       </c>
     </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A81" s="1">
         <v>36770</v>
       </c>
@@ -1319,7 +1319,7 @@
         <v>26542.167916748</v>
       </c>
     </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A82" s="1">
         <v>36800</v>
       </c>
@@ -1330,7 +1330,7 @@
         <v>25043.483939992399</v>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A83" s="1">
         <v>36831</v>
       </c>
@@ -1341,7 +1341,7 @@
         <v>24995.5922893963</v>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A84" s="1">
         <v>36861</v>
       </c>
@@ -1352,7 +1352,7 @@
         <v>27620.319277143401</v>
       </c>
     </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A85" s="1">
         <v>36892</v>
       </c>
@@ -1363,7 +1363,7 @@
         <v>24612.0005935267</v>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A86" s="1">
         <v>36923</v>
       </c>
@@ -1374,7 +1374,7 @@
         <v>19274.859027923801</v>
       </c>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A87" s="1">
         <v>36951</v>
       </c>
@@ -1385,7 +1385,7 @@
         <v>23731.055231634899</v>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A88" s="1">
         <v>36982</v>
       </c>
@@ -1396,7 +1396,7 @@
         <v>24375.407581475902</v>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A89" s="1">
         <v>37012</v>
       </c>
@@ -1407,7 +1407,7 @@
         <v>23883.207074048601</v>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A90" s="1">
         <v>37043</v>
       </c>
@@ -1418,7 +1418,7 @@
         <v>23044.011165833599</v>
       </c>
     </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A91" s="1">
         <v>37073</v>
       </c>
@@ -1429,7 +1429,7 @@
         <v>20871.218348611001</v>
       </c>
     </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A92" s="1">
         <v>37104</v>
       </c>
@@ -1440,7 +1440,7 @@
         <v>14056.847280329301</v>
       </c>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A93" s="1">
         <v>37135</v>
       </c>
@@ -1451,7 +1451,7 @@
         <v>15018.533105483801</v>
       </c>
     </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A94" s="1">
         <v>37165</v>
       </c>
@@ -1462,7 +1462,7 @@
         <v>13946.766587329899</v>
       </c>
     </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A95" s="1">
         <v>37196</v>
       </c>
@@ -1473,7 +1473,7 @@
         <v>12802.930420660001</v>
       </c>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A96" s="1">
         <v>37226</v>
       </c>
@@ -1484,7 +1484,7 @@
         <v>11193.117448711901</v>
       </c>
     </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A97" s="1">
         <v>37257</v>
       </c>
@@ -1495,7 +1495,7 @@
         <v>16697.178628423499</v>
       </c>
     </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A98" s="1">
         <v>37288</v>
       </c>
@@ -1506,7 +1506,7 @@
         <v>11637.0059091123</v>
       </c>
     </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A99" s="1">
         <v>37316</v>
       </c>
@@ -1517,7 +1517,7 @@
         <v>11629.965782556599</v>
       </c>
     </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A100" s="1">
         <v>37347</v>
       </c>
@@ -1528,7 +1528,7 @@
         <v>13109.3279377947</v>
       </c>
     </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A101" s="1">
         <v>37377</v>
       </c>
@@ -1539,7 +1539,7 @@
         <v>11229.1688365022</v>
       </c>
     </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A102" s="1">
         <v>37408</v>
       </c>
@@ -1550,7 +1550,7 @@
         <v>13196.9484592188</v>
       </c>
     </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A103" s="1">
         <v>37438</v>
       </c>
@@ -1561,7 +1561,7 @@
         <v>12176.1961354264</v>
       </c>
     </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A104" s="1">
         <v>37469</v>
       </c>
@@ -1572,7 +1572,7 @@
         <v>12317.288272924399</v>
       </c>
     </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A105" s="1">
         <v>37500</v>
       </c>
@@ -1583,7 +1583,7 @@
         <v>12865.4061426927</v>
       </c>
     </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A106" s="1">
         <v>37530</v>
       </c>
@@ -1594,7 +1594,7 @@
         <v>11661.005275199601</v>
       </c>
     </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A107" s="1">
         <v>37561</v>
       </c>
@@ -1605,7 +1605,7 @@
         <v>12123.5078203261</v>
       </c>
     </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A108" s="1">
         <v>37591</v>
       </c>
@@ -1616,7 +1616,7 @@
         <v>13781.7390091367</v>
       </c>
     </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A109" s="1">
         <v>37622</v>
       </c>
@@ -1627,7 +1627,7 @@
         <v>20918.3111980182</v>
       </c>
     </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A110" s="1">
         <v>37653</v>
       </c>
@@ -1638,7 +1638,7 @@
         <v>13013.180399668699</v>
       </c>
     </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A111" s="1">
         <v>37681</v>
       </c>
@@ -1649,7 +1649,7 @@
         <v>13488.9149745467</v>
       </c>
     </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A112" s="1">
         <v>37712</v>
       </c>
@@ -1660,7 +1660,7 @@
         <v>11988.7286223226</v>
       </c>
     </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A113" s="1">
         <v>37742</v>
       </c>
@@ -1671,7 +1671,7 @@
         <v>11872.7840869878</v>
       </c>
     </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A114" s="1">
         <v>37773</v>
       </c>
@@ -1682,7 +1682,7 @@
         <v>11761.436808263699</v>
       </c>
     </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A115" s="1">
         <v>37803</v>
       </c>
@@ -1693,7 +1693,7 @@
         <v>8679.9450308908908</v>
       </c>
     </row>
-    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A116" s="1">
         <v>37834</v>
       </c>
@@ -1704,7 +1704,7 @@
         <v>13721.0718563505</v>
       </c>
     </row>
-    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A117" s="1">
         <v>37865</v>
       </c>
@@ -1715,7 +1715,7 @@
         <v>11728.8977731627</v>
       </c>
     </row>
-    <row r="118" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A118" s="1">
         <v>37895</v>
       </c>
@@ -1726,7 +1726,7 @@
         <v>11775.9687061809</v>
       </c>
     </row>
-    <row r="119" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A119" s="1">
         <v>37926</v>
       </c>
@@ -1737,7 +1737,7 @@
         <v>15889.7751105641</v>
       </c>
     </row>
-    <row r="120" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A120" s="1">
         <v>37956</v>
       </c>
@@ -1748,7 +1748,7 @@
         <v>13864.427280611801</v>
       </c>
     </row>
-    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A121" s="1">
         <v>37987</v>
       </c>
@@ -1759,7 +1759,7 @@
         <v>26059.378509985301</v>
       </c>
     </row>
-    <row r="122" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A122" s="1">
         <v>38018</v>
       </c>
@@ -1770,7 +1770,7 @@
         <v>19675.098733004801</v>
       </c>
     </row>
-    <row r="123" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A123" s="1">
         <v>38047</v>
       </c>
@@ -1781,7 +1781,7 @@
         <v>17916.848891443198</v>
       </c>
     </row>
-    <row r="124" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A124" s="1">
         <v>38078</v>
       </c>
@@ -1792,7 +1792,7 @@
         <v>16768.522190977201</v>
       </c>
     </row>
-    <row r="125" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A125" s="1">
         <v>38108</v>
       </c>
@@ -1803,7 +1803,7 @@
         <v>20458.413408075699</v>
       </c>
     </row>
-    <row r="126" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A126" s="1">
         <v>38139</v>
       </c>
@@ -1814,7 +1814,7 @@
         <v>18677.229180470898</v>
       </c>
     </row>
-    <row r="127" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A127" s="1">
         <v>38169</v>
       </c>
@@ -1825,7 +1825,7 @@
         <v>18691.2440998948</v>
       </c>
     </row>
-    <row r="128" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A128" s="1">
         <v>38200</v>
       </c>
@@ -1836,7 +1836,7 @@
         <v>19451.2318676219</v>
       </c>
     </row>
-    <row r="129" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A129" s="1">
         <v>38231</v>
       </c>
@@ -1847,7 +1847,7 @@
         <v>20245.247154316399</v>
       </c>
     </row>
-    <row r="130" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A130" s="1">
         <v>38261</v>
       </c>
@@ -1858,7 +1858,7 @@
         <v>22419.924651805199</v>
       </c>
     </row>
-    <row r="131" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A131" s="1">
         <v>38292</v>
       </c>
@@ -1869,7 +1869,7 @@
         <v>20802.394650128099</v>
       </c>
     </row>
-    <row r="132" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A132" s="1">
         <v>38322</v>
       </c>
@@ -1880,7 +1880,7 @@
         <v>22616.029191390098</v>
       </c>
     </row>
-    <row r="133" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A133" s="1">
         <v>38353</v>
       </c>
@@ -1891,7 +1891,7 @@
         <v>37786.773146772597</v>
       </c>
     </row>
-    <row r="134" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A134" s="1">
         <v>38384</v>
       </c>
@@ -1902,7 +1902,7 @@
         <v>15480.416353570899</v>
       </c>
     </row>
-    <row r="135" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A135" s="1">
         <v>38412</v>
       </c>
@@ -1913,7 +1913,7 @@
         <v>23666.288895595299</v>
       </c>
     </row>
-    <row r="136" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A136" s="1">
         <v>38443</v>
       </c>
@@ -1924,7 +1924,7 @@
         <v>25570.910457669299</v>
       </c>
     </row>
-    <row r="137" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A137" s="1">
         <v>38473</v>
       </c>
@@ -1935,7 +1935,7 @@
         <v>24391.915198571201</v>
       </c>
     </row>
-    <row r="138" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A138" s="1">
         <v>38504</v>
       </c>
@@ -1946,7 +1946,7 @@
         <v>23139.706424755601</v>
       </c>
     </row>
-    <row r="139" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A139" s="1">
         <v>38534</v>
       </c>
@@ -1957,7 +1957,7 @@
         <v>26000.6527916913</v>
       </c>
     </row>
-    <row r="140" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A140" s="1">
         <v>38565</v>
       </c>
@@ -1968,7 +1968,7 @@
         <v>23274.602771414298</v>
       </c>
     </row>
-    <row r="141" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A141" s="1">
         <v>38596</v>
       </c>
@@ -1979,7 +1979,7 @@
         <v>22574.956124004599</v>
       </c>
     </row>
-    <row r="142" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A142" s="1">
         <v>38626</v>
       </c>
@@ -1990,7 +1990,7 @@
         <v>25984.4902371842</v>
       </c>
     </row>
-    <row r="143" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A143" s="1">
         <v>38657</v>
       </c>
@@ -2001,7 +2001,7 @@
         <v>26351.159770474998</v>
       </c>
     </row>
-    <row r="144" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A144" s="1">
         <v>38687</v>
       </c>
@@ -2012,7 +2012,7 @@
         <v>23783.133059075099</v>
       </c>
     </row>
-    <row r="145" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A145" s="1">
         <v>38718</v>
       </c>
@@ -2023,7 +2023,7 @@
         <v>27915.8810871032</v>
       </c>
     </row>
-    <row r="146" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A146" s="1">
         <v>38749</v>
       </c>
@@ -2034,7 +2034,7 @@
         <v>32139.051187794201</v>
       </c>
     </row>
-    <row r="147" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A147" s="1">
         <v>38777</v>
       </c>
@@ -2045,7 +2045,7 @@
         <v>30711.838740336301</v>
       </c>
     </row>
-    <row r="148" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A148" s="1">
         <v>38808</v>
       </c>
@@ -2056,7 +2056,7 @@
         <v>33189.707869465201</v>
       </c>
     </row>
-    <row r="149" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A149" s="1">
         <v>38838</v>
       </c>
@@ -2067,7 +2067,7 @@
         <v>27489.554126411502</v>
       </c>
     </row>
-    <row r="150" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A150" s="1">
         <v>38869</v>
       </c>
@@ -2078,7 +2078,7 @@
         <v>31945.162791823099</v>
       </c>
     </row>
-    <row r="151" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A151" s="1">
         <v>38899</v>
       </c>
@@ -2089,7 +2089,7 @@
         <v>35465.725548441202</v>
       </c>
     </row>
-    <row r="152" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A152" s="1">
         <v>38930</v>
       </c>
@@ -2100,7 +2100,7 @@
         <v>34274.995692589</v>
       </c>
     </row>
-    <row r="153" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A153" s="1">
         <v>38961</v>
       </c>
@@ -2111,7 +2111,7 @@
         <v>37775.2420417744</v>
       </c>
     </row>
-    <row r="154" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A154" s="1">
         <v>38991</v>
       </c>
@@ -2122,7 +2122,7 @@
         <v>35778.523380069797</v>
       </c>
     </row>
-    <row r="155" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A155" s="1">
         <v>39022</v>
       </c>
@@ -2133,7 +2133,7 @@
         <v>39261.673015845103</v>
       </c>
     </row>
-    <row r="156" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A156" s="1">
         <v>39052</v>
       </c>
@@ -2144,7 +2144,7 @@
         <v>41654.965002240497</v>
       </c>
     </row>
-    <row r="157" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A157" s="1">
         <v>39083</v>
       </c>
@@ -2155,7 +2155,7 @@
         <v>31733.618236988899</v>
       </c>
     </row>
-    <row r="158" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A158" s="1">
         <v>39114</v>
       </c>
@@ -2166,7 +2166,7 @@
         <v>40023.961094888298</v>
       </c>
     </row>
-    <row r="159" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A159" s="1">
         <v>39142</v>
       </c>
@@ -2177,7 +2177,7 @@
         <v>43055.6998839894</v>
       </c>
     </row>
-    <row r="160" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A160" s="1">
         <v>39173</v>
       </c>
@@ -2188,7 +2188,7 @@
         <v>39573.272201158499</v>
       </c>
     </row>
-    <row r="161" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A161" s="1">
         <v>39203</v>
       </c>
@@ -2199,7 +2199,7 @@
         <v>40544.565717479803</v>
       </c>
     </row>
-    <row r="162" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A162" s="1">
         <v>39234</v>
       </c>
@@ -2210,7 +2210,7 @@
         <v>44575.540738497002</v>
       </c>
     </row>
-    <row r="163" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A163" s="1">
         <v>39264</v>
       </c>
@@ -2221,7 +2221,7 @@
         <v>39298.085868881702</v>
       </c>
     </row>
-    <row r="164" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A164" s="1">
         <v>39295</v>
       </c>
@@ -2232,7 +2232,7 @@
         <v>44075.936516071502</v>
       </c>
     </row>
-    <row r="165" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A165" s="1">
         <v>39326</v>
       </c>
@@ -2243,7 +2243,7 @@
         <v>42980.189509053598</v>
       </c>
     </row>
-    <row r="166" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A166" s="1">
         <v>39356</v>
       </c>
@@ -2254,7 +2254,7 @@
         <v>45158.549201938898</v>
       </c>
     </row>
-    <row r="167" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A167" s="1">
         <v>39387</v>
       </c>
@@ -2265,7 +2265,7 @@
         <v>48998.345811177103</v>
       </c>
     </row>
-    <row r="168" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A168" s="1">
         <v>39417</v>
       </c>
@@ -2276,7 +2276,7 @@
         <v>50614.032158375601</v>
       </c>
     </row>
-    <row r="169" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A169" s="1">
         <v>39448</v>
       </c>
@@ -2287,7 +2287,7 @@
         <v>56189.9676900841</v>
       </c>
     </row>
-    <row r="170" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A170" s="1">
         <v>39479</v>
       </c>
@@ -2298,7 +2298,7 @@
         <v>39727.840023930199</v>
       </c>
     </row>
-    <row r="171" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A171" s="1">
         <v>39508</v>
       </c>
@@ -2309,7 +2309,7 @@
         <v>48533.259312729002</v>
       </c>
     </row>
-    <row r="172" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A172" s="1">
         <v>39539</v>
       </c>
@@ -2320,7 +2320,7 @@
         <v>50610.474400491898</v>
       </c>
     </row>
-    <row r="173" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A173" s="1">
         <v>39569</v>
       </c>
@@ -2331,7 +2331,7 @@
         <v>50511.838149394498</v>
       </c>
     </row>
-    <row r="174" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A174" s="1">
         <v>39600</v>
       </c>
@@ -2342,7 +2342,7 @@
         <v>45942.401310522902</v>
       </c>
     </row>
-    <row r="175" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A175" s="1">
         <v>39630</v>
       </c>
@@ -2353,7 +2353,7 @@
         <v>55154.2325168596</v>
       </c>
     </row>
-    <row r="176" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A176" s="1">
         <v>39661</v>
       </c>
@@ -2364,7 +2364,7 @@
         <v>49866.952214057303</v>
       </c>
     </row>
-    <row r="177" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A177" s="1">
         <v>39692</v>
       </c>
@@ -2375,7 +2375,7 @@
         <v>50486.126568428102</v>
       </c>
     </row>
-    <row r="178" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A178" s="1">
         <v>39722</v>
       </c>
@@ -2386,7 +2386,7 @@
         <v>46951.234543487502</v>
       </c>
     </row>
-    <row r="179" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A179" s="1">
         <v>39753</v>
       </c>
@@ -2397,7 +2397,7 @@
         <v>35503.155229219497</v>
       </c>
     </row>
-    <row r="180" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A180" s="1">
         <v>39783</v>
       </c>
@@ -2408,7 +2408,7 @@
         <v>26849.5848447879</v>
       </c>
     </row>
-    <row r="181" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A181" s="1">
         <v>39814</v>
       </c>
@@ -2419,7 +2419,7 @@
         <v>37125.112203779303</v>
       </c>
     </row>
-    <row r="182" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A182" s="1">
         <v>39845</v>
       </c>
@@ -2430,7 +2430,7 @@
         <v>22666.364942668799</v>
       </c>
     </row>
-    <row r="183" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A183" s="1">
         <v>39873</v>
       </c>
@@ -2441,7 +2441,7 @@
         <v>38095.498652472299</v>
       </c>
     </row>
-    <row r="184" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A184" s="1">
         <v>39904</v>
       </c>
@@ -2452,7 +2452,7 @@
         <v>36960.380828133297</v>
       </c>
     </row>
-    <row r="185" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A185" s="1">
         <v>39934</v>
       </c>
@@ -2463,7 +2463,7 @@
         <v>41045.180362297702</v>
       </c>
     </row>
-    <row r="186" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A186" s="1">
         <v>39965</v>
       </c>
@@ -2474,7 +2474,7 @@
         <v>39684.006114346499</v>
       </c>
     </row>
-    <row r="187" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A187" s="1">
         <v>39995</v>
       </c>
@@ -2485,7 +2485,7 @@
         <v>43450.119366890503</v>
       </c>
     </row>
-    <row r="188" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A188" s="1">
         <v>40026</v>
       </c>
@@ -2496,7 +2496,7 @@
         <v>41242.4833607029</v>
       </c>
     </row>
-    <row r="189" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A189" s="1">
         <v>40057</v>
       </c>
@@ -2507,7 +2507,7 @@
         <v>44831.3100880696</v>
       </c>
     </row>
-    <row r="190" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A190" s="1">
         <v>40087</v>
       </c>
@@ -2518,7 +2518,7 @@
         <v>49196.509532347198</v>
       </c>
     </row>
-    <row r="191" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A191" s="1">
         <v>40118</v>
       </c>
@@ -2529,7 +2529,7 @@
         <v>49481.486636896101</v>
       </c>
     </row>
-    <row r="192" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A192" s="1">
         <v>40148</v>
       </c>
@@ -2540,7 +2540,7 @@
         <v>53632.493010406797</v>
       </c>
     </row>
-    <row r="193" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A193" s="1">
         <v>40179</v>
       </c>
@@ -2551,7 +2551,7 @@
         <v>52177.008498281102</v>
       </c>
     </row>
-    <row r="194" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A194" s="1">
         <v>40210</v>
       </c>
@@ -2562,7 +2562,7 @@
         <v>47846.591119550001</v>
       </c>
     </row>
-    <row r="195" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A195" s="1">
         <v>40238</v>
       </c>
@@ -2573,7 +2573,7 @@
         <v>49800.049537067098</v>
       </c>
     </row>
-    <row r="196" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A196" s="1">
         <v>40269</v>
       </c>
@@ -2584,7 +2584,7 @@
         <v>55605.559642491498</v>
       </c>
     </row>
-    <row r="197" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A197" s="1">
         <v>40299</v>
       </c>
@@ -2595,7 +2595,7 @@
         <v>56864.860591375502</v>
       </c>
     </row>
-    <row r="198" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A198" s="1">
         <v>40330</v>
       </c>
@@ -2606,7 +2606,7 @@
         <v>58826.211827195897</v>
       </c>
     </row>
-    <row r="199" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A199" s="1">
         <v>40360</v>
       </c>
@@ -2617,7 +2617,7 @@
         <v>54883.807455357302</v>
       </c>
     </row>
-    <row r="200" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A200" s="1">
         <v>40391</v>
       </c>
@@ -2628,7 +2628,7 @@
         <v>62626.5571456873</v>
       </c>
     </row>
-    <row r="201" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A201" s="1">
         <v>40422</v>
       </c>
@@ -2639,7 +2639,7 @@
         <v>62746.1358972991</v>
       </c>
     </row>
-    <row r="202" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A202" s="1">
         <v>40452</v>
       </c>
@@ -2650,7 +2650,7 @@
         <v>59328.149172613899</v>
       </c>
     </row>
-    <row r="203" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A203" s="1">
         <v>40483</v>
       </c>
@@ -2661,7 +2661,7 @@
         <v>66681.299492051898</v>
       </c>
     </row>
-    <row r="204" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A204" s="1">
         <v>40513</v>
       </c>
@@ -2672,7 +2672,7 @@
         <v>68065.963044230797</v>
       </c>
     </row>
-    <row r="205" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A205" s="1">
         <v>40544</v>
       </c>
@@ -2683,7 +2683,7 @@
         <v>68522.225555524899</v>
       </c>
     </row>
-    <row r="206" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A206" s="1">
         <v>40575</v>
       </c>
@@ -2694,7 +2694,7 @@
         <v>48896.347904593502</v>
       </c>
     </row>
-    <row r="207" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A207" s="1">
         <v>40603</v>
       </c>
@@ -2705,7 +2705,7 @@
         <v>66304.091289931195</v>
       </c>
     </row>
-    <row r="208" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A208" s="1">
         <v>40634</v>
       </c>
@@ -2716,7 +2716,7 @@
         <v>72152.876938262605</v>
       </c>
     </row>
-    <row r="209" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A209" s="1">
         <v>40664</v>
       </c>
@@ -2727,7 +2727,7 @@
         <v>74778.828326602903</v>
       </c>
     </row>
-    <row r="210" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A210" s="1">
         <v>40695</v>
       </c>
@@ -2738,7 +2738,7 @@
         <v>74437.213815002295</v>
       </c>
     </row>
-    <row r="211" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A211" s="1">
         <v>40725</v>
       </c>
@@ -2749,7 +2749,7 @@
         <v>69418.473099511801</v>
       </c>
     </row>
-    <row r="212" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A212" s="1">
         <v>40756</v>
       </c>
@@ -2760,7 +2760,7 @@
         <v>73346.200616379094</v>
       </c>
     </row>
-    <row r="213" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A213" s="1">
         <v>40787</v>
       </c>
@@ -2771,7 +2771,7 @@
         <v>69216.682459980104</v>
       </c>
     </row>
-    <row r="214" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A214" s="1">
         <v>40817</v>
       </c>
@@ -2782,7 +2782,7 @@
         <v>65761.865254955206</v>
       </c>
     </row>
-    <row r="215" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A215" s="1">
         <v>40848</v>
       </c>
@@ -2793,7 +2793,7 @@
         <v>65671.560630246997</v>
       </c>
     </row>
-    <row r="216" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A216" s="1">
         <v>40878</v>
       </c>
@@ -2804,7 +2804,7 @@
         <v>57677.023248363599</v>
       </c>
     </row>
-    <row r="217" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A217" s="1">
         <v>40909</v>
       </c>
@@ -2815,7 +2815,7 @@
         <v>63078.104760717899</v>
       </c>
     </row>
-    <row r="218" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A218" s="1">
         <v>40940</v>
       </c>
@@ -2826,7 +2826,7 @@
         <v>62420.809958065998</v>
       </c>
     </row>
-    <row r="219" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A219" s="1">
         <v>40969</v>
       </c>
@@ -2837,7 +2837,7 @@
         <v>63934.098328846398</v>
       </c>
     </row>
-    <row r="220" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A220" s="1">
         <v>41000</v>
       </c>
@@ -2848,7 +2848,7 @@
         <v>54277.236216549201</v>
       </c>
     </row>
-    <row r="221" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A221" s="1">
         <v>41030</v>
       </c>
@@ -2859,7 +2859,7 @@
         <v>53952.307373920601</v>
       </c>
     </row>
-    <row r="222" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A222" s="1">
         <v>41061</v>
       </c>
@@ -2870,7 +2870,7 @@
         <v>48405.416421620997</v>
       </c>
     </row>
-    <row r="223" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A223" s="1">
         <v>41091</v>
       </c>
@@ -2881,7 +2881,7 @@
         <v>63522.836910316801</v>
       </c>
     </row>
-    <row r="224" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A224" s="1">
         <v>41122</v>
       </c>
@@ -2892,7 +2892,7 @@
         <v>69585.760496837</v>
       </c>
     </row>
-    <row r="225" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A225" s="1">
         <v>41153</v>
       </c>
@@ -2903,7 +2903,7 @@
         <v>61285.047127898702</v>
       </c>
     </row>
-    <row r="226" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A226" s="1">
         <v>41183</v>
       </c>
@@ -2914,7 +2914,7 @@
         <v>68186.528893732902</v>
       </c>
     </row>
-    <row r="227" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A227" s="1">
         <v>41214</v>
       </c>
@@ -2925,7 +2925,7 @@
         <v>68924.465717758299</v>
       </c>
     </row>
-    <row r="228" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A228" s="1">
         <v>41244</v>
       </c>
@@ -2936,7 +2936,7 @@
         <v>69692.333113065499</v>
       </c>
     </row>
-    <row r="229" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A229" s="1">
         <v>41275</v>
       </c>
@@ -2947,7 +2947,7 @@
         <v>64172.674516478502</v>
       </c>
     </row>
-    <row r="230" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A230" s="1">
         <v>41306</v>
       </c>
@@ -2958,7 +2958,7 @@
         <v>57168.754010554097</v>
       </c>
     </row>
-    <row r="231" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A231" s="1">
         <v>41334</v>
       </c>
@@ -2969,7 +2969,7 @@
         <v>74124.896164676</v>
       </c>
     </row>
-    <row r="232" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A232" s="1">
         <v>41365</v>
       </c>
@@ -2980,7 +2980,7 @@
         <v>71624.111919594405</v>
       </c>
     </row>
-    <row r="233" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A233" s="1">
         <v>41395</v>
       </c>
@@ -2991,7 +2991,7 @@
         <v>73695.472691965493</v>
       </c>
     </row>
-    <row r="234" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A234" s="1">
         <v>41426</v>
       </c>
@@ -3002,7 +3002,7 @@
         <v>59699.220254849301</v>
       </c>
     </row>
-    <row r="235" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A235" s="1">
         <v>41456</v>
       </c>
@@ -3013,7 +3013,7 @@
         <v>67938.895501803097</v>
       </c>
     </row>
-    <row r="236" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A236" s="1">
         <v>41487</v>
       </c>
@@ -3024,7 +3024,7 @@
         <v>61954.315246722501</v>
       </c>
     </row>
-    <row r="237" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A237" s="1">
         <v>41518</v>
       </c>
@@ -3035,7 +3035,7 @@
         <v>62964.707547203398</v>
       </c>
     </row>
-    <row r="238" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A238" s="1">
         <v>41548</v>
       </c>
@@ -3046,7 +3046,7 @@
         <v>64145.121291411597</v>
       </c>
     </row>
-    <row r="239" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A239" s="1">
         <v>41579</v>
       </c>
@@ -3057,7 +3057,7 @@
         <v>54606.939123789001</v>
       </c>
     </row>
-    <row r="240" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A240" s="1">
         <v>41609</v>
       </c>
@@ -3068,7 +3068,7 @@
         <v>52588.293010538699</v>
       </c>
     </row>
-    <row r="241" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A241" s="1">
         <v>41640</v>
       </c>
@@ -3079,7 +3079,7 @@
         <v>56249.516796244403</v>
       </c>
     </row>
-    <row r="242" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A242" s="1">
         <v>41671</v>
       </c>
@@ -3090,7 +3090,7 @@
         <v>55469.5812377486</v>
       </c>
     </row>
-    <row r="243" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A243" s="1">
         <v>41699</v>
       </c>
@@ -3101,7 +3101,7 @@
         <v>52975.954074941401</v>
       </c>
     </row>
-    <row r="244" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A244" s="1">
         <v>41730</v>
       </c>
@@ -3112,7 +3112,7 @@
         <v>54942.343159671997</v>
       </c>
     </row>
-    <row r="245" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A245" s="1">
         <v>41760</v>
       </c>
@@ -3123,7 +3123,7 @@
         <v>47341.610484953599</v>
       </c>
     </row>
-    <row r="246" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A246" s="1">
         <v>41791</v>
       </c>
@@ -3134,7 +3134,7 @@
         <v>45950.527460567602</v>
       </c>
     </row>
-    <row r="247" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A247" s="1">
         <v>41821</v>
       </c>
@@ -3145,7 +3145,7 @@
         <v>45779.437032580303</v>
       </c>
     </row>
-    <row r="248" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A248" s="1">
         <v>41852</v>
       </c>
@@ -3156,7 +3156,7 @@
         <v>41820.492136728099</v>
       </c>
     </row>
-    <row r="249" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A249" s="1">
         <v>41883</v>
       </c>
@@ -3167,7 +3167,7 @@
         <v>48498.062017315999</v>
       </c>
     </row>
-    <row r="250" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A250" s="1">
         <v>41913</v>
       </c>
@@ -3178,7 +3178,7 @@
         <v>50522.355539148601</v>
       </c>
     </row>
-    <row r="251" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A251" s="1">
         <v>41944</v>
       </c>
@@ -3189,7 +3189,7 @@
         <v>49569.448687346303</v>
       </c>
     </row>
-    <row r="252" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A252" s="1">
         <v>41974</v>
       </c>
@@ -3200,7 +3200,7 @@
         <v>48109.852492785503</v>
       </c>
     </row>
-    <row r="253" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A253" s="1">
         <v>42005</v>
       </c>
@@ -3211,7 +3211,7 @@
         <v>47063.637704828303</v>
       </c>
     </row>
-    <row r="254" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A254" s="1">
         <v>42036</v>
       </c>
@@ -3222,7 +3222,7 @@
         <v>48021.251063788302</v>
       </c>
     </row>
-    <row r="255" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A255" s="1">
         <v>42064</v>
       </c>
@@ -3233,7 +3233,7 @@
         <v>45580.634610757603</v>
       </c>
     </row>
-    <row r="256" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A256" s="1">
         <v>42095</v>
       </c>
@@ -3244,7 +3244,7 @@
         <v>41576.2947299718</v>
       </c>
     </row>
-    <row r="257" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A257" s="1">
         <v>42125</v>
       </c>
@@ -3255,7 +3255,7 @@
         <v>43793.297231736702</v>
       </c>
     </row>
-    <row r="258" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A258" s="1">
         <v>42156</v>
       </c>
@@ -3266,7 +3266,7 @@
         <v>47738.857295376903</v>
       </c>
     </row>
-    <row r="259" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A259" s="1">
         <v>42186</v>
       </c>
@@ -3277,7 +3277,7 @@
         <v>42074.174519223103</v>
       </c>
     </row>
-    <row r="260" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A260" s="1">
         <v>42217</v>
       </c>
@@ -3288,7 +3288,7 @@
         <v>45232.600555774399</v>
       </c>
     </row>
-    <row r="261" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A261" s="1">
         <v>42248</v>
       </c>
@@ -3299,7 +3299,7 @@
         <v>45563.371394408801</v>
       </c>
     </row>
-    <row r="262" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A262" s="1">
         <v>42278</v>
       </c>
@@ -3310,7 +3310,7 @@
         <v>39424.1490164715</v>
       </c>
     </row>
-    <row r="263" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A263" s="1">
         <v>42309</v>
       </c>
@@ -3321,7 +3321,7 @@
         <v>40919.253118666798</v>
       </c>
     </row>
-    <row r="264" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A264" s="1">
         <v>42339</v>
       </c>
@@ -3332,7 +3332,7 @@
         <v>39707.597566322402</v>
       </c>
     </row>
-    <row r="265" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A265" s="1">
         <v>42370</v>
       </c>
@@ -3343,7 +3343,7 @@
         <v>40460.781695048601</v>
       </c>
     </row>
-    <row r="266" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A266" s="1">
         <v>42401</v>
       </c>
@@ -3354,7 +3354,7 @@
         <v>38655.118842960699</v>
       </c>
     </row>
-    <row r="267" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A267" s="1">
         <v>42430</v>
       </c>
@@ -3365,7 +3365,7 @@
         <v>40376.524819804203</v>
       </c>
     </row>
-    <row r="268" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A268" s="1">
         <v>42461</v>
       </c>
@@ -3376,7 +3376,7 @@
         <v>42538.368185861204</v>
       </c>
     </row>
-    <row r="269" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A269" s="1">
         <v>42491</v>
       </c>
@@ -3387,7 +3387,7 @@
         <v>37613.9004032343</v>
       </c>
     </row>
-    <row r="270" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A270" s="1">
         <v>42522</v>
       </c>
@@ -3398,7 +3398,7 @@
         <v>37662.447275230901</v>
       </c>
     </row>
-    <row r="271" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A271" s="1">
         <v>42552</v>
       </c>
@@ -3409,7 +3409,7 @@
         <v>39775.644562766298</v>
       </c>
     </row>
-    <row r="272" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A272" s="1">
         <v>42583</v>
       </c>
@@ -3420,7 +3420,7 @@
         <v>37728.136504122303</v>
       </c>
     </row>
-    <row r="273" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A273" s="1">
         <v>42614</v>
       </c>
@@ -3431,7 +3431,7 @@
         <v>35648.701492859604</v>
       </c>
     </row>
-    <row r="274" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A274" s="1">
         <v>42644</v>
       </c>
@@ -3442,7 +3442,7 @@
         <v>34703.734362406001</v>
       </c>
     </row>
-    <row r="275" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A275" s="1">
         <v>42675</v>
       </c>
@@ -3453,7 +3453,7 @@
         <v>41436.256786474798</v>
       </c>
     </row>
-    <row r="276" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A276" s="1">
         <v>42705</v>
       </c>
@@ -3464,7 +3464,7 @@
         <v>49299.512380953798</v>
       </c>
     </row>
-    <row r="277" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A277" s="1">
         <v>42736</v>
       </c>
@@ -3475,7 +3475,7 @@
         <v>47083.855090298799</v>
       </c>
     </row>
-    <row r="278" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A278" s="1">
         <v>42767</v>
       </c>
@@ -3486,7 +3486,7 @@
         <v>27846.650832241699</v>
       </c>
     </row>
-    <row r="279" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A279" s="1">
         <v>42795</v>
       </c>
@@ -3497,7 +3497,7 @@
         <v>33784.569384668299</v>
       </c>
     </row>
-    <row r="280" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A280" s="1">
         <v>42826</v>
       </c>
@@ -3508,7 +3508,7 @@
         <v>37293.457117649603</v>
       </c>
     </row>
-    <row r="281" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A281" s="1">
         <v>42856</v>
       </c>
@@ -3519,7 +3519,7 @@
         <v>41725.087326745903</v>
       </c>
     </row>
-    <row r="282" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A282" s="1">
         <v>42887</v>
       </c>
@@ -3530,7 +3530,7 @@
         <v>42323.181843003098</v>
       </c>
     </row>
-    <row r="283" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A283" s="1">
         <v>42917</v>
       </c>
@@ -3541,7 +3541,7 @@
         <v>40235.427356639397</v>
       </c>
     </row>
-    <row r="284" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A284" s="1">
         <v>42948</v>
       </c>
@@ -3552,7 +3552,7 @@
         <v>38556.522531382601</v>
       </c>
     </row>
-    <row r="285" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A285" s="1">
         <v>42979</v>
       </c>
@@ -3563,7 +3563,7 @@
         <v>42303.373330175396</v>
       </c>
     </row>
-    <row r="286" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A286" s="1">
         <v>43009</v>
       </c>
@@ -3574,7 +3574,7 @@
         <v>40153.996453462001</v>
       </c>
     </row>
-    <row r="287" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A287" s="1">
         <v>43040</v>
       </c>
@@ -3585,7 +3585,7 @@
         <v>40070.523544119103</v>
       </c>
     </row>
-    <row r="288" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A288" s="1">
         <v>43070</v>
       </c>
@@ -3596,7 +3596,7 @@
         <v>43107.672629774497</v>
       </c>
     </row>
-    <row r="289" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A289" s="1">
         <v>43101</v>
       </c>
@@ -3607,7 +3607,7 @@
         <v>40120.2864482597</v>
       </c>
     </row>
-    <row r="290" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A290" s="1">
         <v>43132</v>
       </c>
@@ -3618,7 +3618,7 @@
         <v>40492.263143173397</v>
       </c>
     </row>
-    <row r="291" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A291" s="1">
         <v>43160</v>
       </c>
@@ -3629,7 +3629,7 @@
         <v>45072.924012819203</v>
       </c>
     </row>
-    <row r="292" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A292" s="1">
         <v>43191</v>
       </c>
@@ -3640,7 +3640,7 @@
         <v>44474.568777107801</v>
       </c>
     </row>
-    <row r="293" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A293" s="1">
         <v>43221</v>
       </c>
@@ -3651,7 +3651,7 @@
         <v>43253.639566649697</v>
       </c>
     </row>
-    <row r="294" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A294" s="1">
         <v>43252</v>
       </c>
@@ -3662,7 +3662,7 @@
         <v>38189.213565880898</v>
       </c>
     </row>
-    <row r="295" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A295" s="1">
         <v>43282</v>
       </c>
@@ -3673,7 +3673,7 @@
         <v>42331.740908612002</v>
       </c>
     </row>
-    <row r="296" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A296" s="1">
         <v>43313</v>
       </c>
@@ -3684,7 +3684,7 @@
         <v>42271.359310453998</v>
       </c>
     </row>
-    <row r="297" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A297" s="1">
         <v>43344</v>
       </c>
@@ -3695,7 +3695,7 @@
         <v>34354.952037385898</v>
       </c>
     </row>
-    <row r="298" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A298" s="1">
         <v>43374</v>
       </c>
@@ -3706,7 +3706,7 @@
         <v>33806.211249831598</v>
       </c>
     </row>
-    <row r="299" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A299" s="1">
         <v>43405</v>
       </c>
@@ -3717,7 +3717,7 @@
         <v>32087.091302744699</v>
       </c>
     </row>
-    <row r="300" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A300" s="1">
         <v>43435</v>
       </c>
@@ -3728,7 +3728,7 @@
         <v>29337.705828173101</v>
       </c>
     </row>
-    <row r="301" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A301" s="1">
         <v>43466</v>
       </c>
@@ -3739,7 +3739,7 @@
         <v>32774.588345043099</v>
       </c>
     </row>
-    <row r="302" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A302" s="1">
         <v>43497</v>
       </c>
@@ -3750,7 +3750,7 @@
         <v>33850.969226474801</v>
       </c>
     </row>
-    <row r="303" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A303" s="1">
         <v>43525</v>
       </c>
@@ -3761,7 +3761,7 @@
         <v>25548.491978698199</v>
       </c>
     </row>
-    <row r="304" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A304" s="1">
         <v>43556</v>
       </c>
@@ -3772,7 +3772,7 @@
         <v>27927.395591348599</v>
       </c>
     </row>
-    <row r="305" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A305" s="1">
         <v>43586</v>
       </c>
@@ -3783,7 +3783,7 @@
         <v>27089.717962017501</v>
       </c>
     </row>
-    <row r="306" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A306" s="1">
         <v>43617</v>
       </c>
@@ -3794,7 +3794,7 @@
         <v>24779.707543456399</v>
       </c>
     </row>
-    <row r="307" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A307" s="1">
         <v>43647</v>
       </c>
@@ -3805,7 +3805,7 @@
         <v>21134.8996194182</v>
       </c>
     </row>
-    <row r="308" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A308" s="1">
         <v>43678</v>
       </c>
@@ -3816,7 +3816,7 @@
         <v>25114.7700069733</v>
       </c>
     </row>
-    <row r="309" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A309" s="1">
         <v>43709</v>
       </c>
@@ -3827,7 +3827,7 @@
         <v>23415.840186911999</v>
       </c>
     </row>
-    <row r="310" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A310" s="1">
         <v>43739</v>
       </c>
@@ -3838,7 +3838,7 @@
         <v>26752.4258883976</v>
       </c>
     </row>
-    <row r="311" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A311" s="1">
         <v>43770</v>
       </c>
@@ -3849,7 +3849,7 @@
         <v>23833.081771402001</v>
       </c>
     </row>
-    <row r="312" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A312" s="1">
         <v>43800</v>
       </c>
@@ -3860,7 +3860,7 @@
         <v>21330.0580755542</v>
       </c>
     </row>
-    <row r="313" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A313" s="1">
         <v>43831</v>
       </c>
@@ -3871,7 +3871,7 @@
         <v>38608.406493054797</v>
       </c>
     </row>
-    <row r="314" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A314" s="1">
         <v>43862</v>
       </c>
@@ -3882,7 +3882,7 @@
         <v>30310.956884001302</v>
       </c>
     </row>
-    <row r="315" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A315" s="1">
         <v>43891</v>
       </c>
@@ -3893,7 +3893,7 @@
         <v>13582.5984692403</v>
       </c>
     </row>
-    <row r="316" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A316" s="1">
         <v>43922</v>
       </c>
@@ -3904,7 +3904,7 @@
         <v>-1914.0001145096501</v>
       </c>
     </row>
-    <row r="317" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A317" s="1">
         <v>43952</v>
       </c>
@@ -3915,7 +3915,7 @@
         <v>5091.2720936564001</v>
       </c>
     </row>
-    <row r="318" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A318" s="1">
         <v>43983</v>
       </c>
@@ -3926,7 +3926,7 @@
         <v>13667.817055317901</v>
       </c>
     </row>
-    <row r="319" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A319" s="1">
         <v>44013</v>
       </c>
@@ -3937,7 +3937,7 @@
         <v>21345.999378959201</v>
       </c>
     </row>
-    <row r="320" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A320" s="1">
         <v>44044</v>
       </c>
@@ -3948,7 +3948,7 @@
         <v>21477.507414945499</v>
       </c>
     </row>
-    <row r="321" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A321" s="1">
         <v>44075</v>
       </c>
@@ -3959,7 +3959,7 @@
         <v>26096.396467118899</v>
       </c>
     </row>
-    <row r="322" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A322" s="1">
         <v>44105</v>
       </c>
@@ -3970,7 +3970,7 @@
         <v>24749.429812734801</v>
       </c>
     </row>
-    <row r="323" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A323" s="1">
         <v>44136</v>
       </c>
@@ -3981,7 +3981,7 @@
         <v>28831.749779906801</v>
       </c>
     </row>
-    <row r="324" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A324" s="1">
         <v>44166</v>
       </c>
@@ -3992,7 +3992,7 @@
         <v>35223.133436700497</v>
       </c>
     </row>
-    <row r="325" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A325" s="1">
         <v>44197</v>
       </c>
@@ -4003,7 +4003,7 @@
         <v>45413.615105028402</v>
       </c>
     </row>
-    <row r="326" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A326" s="1">
         <v>44228</v>
       </c>
@@ -4014,7 +4014,7 @@
         <v>23478.666121369399</v>
       </c>
     </row>
-    <row r="327" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A327" s="1">
         <v>44256</v>
       </c>
@@ -4025,7 +4025,7 @@
         <v>35673.916217009697</v>
       </c>
     </row>
-    <row r="328" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A328" s="1">
         <v>44287</v>
       </c>
@@ -4036,7 +4036,7 @@
         <v>27442.235749490701</v>
       </c>
     </row>
-    <row r="329" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A329" s="1">
         <v>44317</v>
       </c>
@@ -4047,7 +4047,7 @@
         <v>36152.087845109803</v>
       </c>
     </row>
-    <row r="330" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A330" s="1">
         <v>44348</v>
       </c>
@@ -4058,7 +4058,7 @@
         <v>38320.995885091703</v>
       </c>
     </row>
-    <row r="331" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A331" s="1">
         <v>44378</v>
       </c>
@@ -4069,7 +4069,7 @@
         <v>33442.837167354897</v>
       </c>
     </row>
-    <row r="332" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="332" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A332" s="1">
         <v>44409</v>
       </c>
@@ -4080,7 +4080,7 @@
         <v>32182.563663560399</v>
       </c>
     </row>
-    <row r="333" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="333" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A333" s="1">
         <v>44440</v>
       </c>
@@ -4091,7 +4091,7 @@
         <v>37259.860517577101</v>
       </c>
     </row>
-    <row r="334" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="334" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A334" s="1">
         <v>44470</v>
       </c>
@@ -4102,7 +4102,7 @@
         <v>38246.507827763096</v>
       </c>
     </row>
-    <row r="335" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="335" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A335" s="1">
         <v>44501</v>
       </c>
@@ -4113,7 +4113,7 @@
         <v>40383.651691895102</v>
       </c>
     </row>
-    <row r="336" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="336" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A336" s="1">
         <v>44531</v>
       </c>
@@ -4124,7 +4124,7 @@
         <v>45038.961460518003</v>
       </c>
     </row>
-    <row r="337" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="337" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A337" s="1">
         <v>44562</v>
       </c>
@@ -4135,7 +4135,7 @@
         <v>39921.622283552897</v>
       </c>
     </row>
-    <row r="338" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="338" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A338" s="1">
         <v>44593</v>
       </c>
@@ -4146,7 +4146,7 @@
         <v>39998.620077954598</v>
       </c>
     </row>
-    <row r="339" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="339" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A339" s="1">
         <v>44621</v>
       </c>
@@ -4157,7 +4157,7 @@
         <v>41305.985370691298</v>
       </c>
     </row>
-    <row r="340" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="340" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A340" s="1">
         <v>44652</v>
       </c>
@@ -4168,7 +4168,7 @@
         <v>43356.952031082401</v>
       </c>
     </row>
-    <row r="341" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="341" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A341" s="1">
         <v>44682</v>
       </c>
@@ -4179,7 +4179,7 @@
         <v>46793.588320271403</v>
       </c>
     </row>
-    <row r="342" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="342" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A342" s="1">
         <v>44713</v>
       </c>
@@ -4190,7 +4190,7 @@
         <v>46552.192449216498</v>
       </c>
     </row>
-    <row r="343" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="343" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A343" s="1">
         <v>44743</v>
       </c>
@@ -4201,7 +4201,7 @@
         <v>47260.109040917901</v>
       </c>
     </row>
-    <row r="344" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="344" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A344" s="1">
         <v>44774</v>
       </c>
@@ -4212,7 +4212,7 @@
         <v>46153.2820321771</v>
       </c>
     </row>
-    <row r="345" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="345" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A345" s="1">
         <v>44805</v>
       </c>
@@ -4223,7 +4223,7 @@
         <v>45450.973769682401</v>
       </c>
     </row>
-    <row r="346" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="346" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A346" s="1">
         <v>44835</v>
       </c>
@@ -4234,7 +4234,7 @@
         <v>49248.7894174596</v>
       </c>
     </row>
-    <row r="347" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="347" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A347" s="1">
         <v>44866</v>
       </c>
@@ -4245,7 +4245,7 @@
         <v>46540.752380901497</v>
       </c>
     </row>
-    <row r="348" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="348" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A348" s="1">
         <v>44896</v>
       </c>
@@ -4256,7 +4256,7 @@
         <v>44201.4524215282</v>
       </c>
     </row>
-    <row r="349" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="349" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A349" s="1">
         <v>44927</v>
       </c>
@@ -4267,7 +4267,7 @@
         <v>46878.651262367799</v>
       </c>
     </row>
-    <row r="350" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="350" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A350" s="1">
         <v>44958</v>
       </c>
@@ -4278,7 +4278,7 @@
         <v>49537.612610959499</v>
       </c>
     </row>
-    <row r="351" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="351" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A351" s="1">
         <v>44986</v>
       </c>
@@ -4289,7 +4289,7 @@
         <v>53867.271897913299</v>
       </c>
     </row>
-    <row r="352" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="352" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A352" s="1">
         <v>45017</v>
       </c>
@@ -4300,7 +4300,7 @@
         <v>55311.888918935903</v>
       </c>
     </row>
-    <row r="353" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="353" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A353" s="1">
         <v>45047</v>
       </c>
@@ -4311,7 +4311,7 @@
         <v>52544.6477722579</v>
       </c>
     </row>
-    <row r="354" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="354" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A354" s="1">
         <v>45078</v>
       </c>
@@ -4322,7 +4322,7 @@
         <v>51800.233222315903</v>
       </c>
     </row>
-    <row r="355" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="355" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A355" s="1">
         <v>45108</v>
       </c>
@@ -4333,7 +4333,7 @@
         <v>52297.394467467202</v>
       </c>
     </row>
-    <row r="356" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="356" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A356" s="1">
         <v>45139</v>
       </c>
@@ -4344,7 +4344,7 @@
         <v>55120.931976665503</v>
       </c>
     </row>
-    <row r="357" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="357" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A357" s="1">
         <v>45170</v>
       </c>
@@ -4355,7 +4355,7 @@
         <v>51251.255095316097</v>
       </c>
     </row>
-    <row r="358" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="358" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A358" s="1">
         <v>45200</v>
       </c>
@@ -4366,7 +4366,7 @@
         <v>46813.240575017197</v>
       </c>
     </row>
-    <row r="359" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="359" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A359" s="1">
         <v>45231</v>
       </c>
@@ -4377,7 +4377,7 @@
         <v>49404.115124356496</v>
       </c>
     </row>
-    <row r="360" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="360" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A360" s="1">
         <v>45261</v>
       </c>
@@ -4388,7 +4388,7 @@
         <v>46325.766141936198</v>
       </c>
     </row>
-    <row r="361" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="361" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A361" s="1">
         <v>45292</v>
       </c>
@@ -4399,7 +4399,7 @@
         <v>40352.068733406697</v>
       </c>
     </row>
-    <row r="362" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="362" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A362" s="1">
         <v>45323</v>
       </c>
@@ -4410,7 +4410,7 @@
         <v>43363.989911834004</v>
       </c>
     </row>
-    <row r="363" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="363" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A363" s="1">
         <v>45352</v>
       </c>
@@ -4421,7 +4421,7 @@
         <v>39250.383915926897</v>
       </c>
     </row>
-    <row r="364" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="364" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A364" s="1">
         <v>45383</v>
       </c>
@@ -4432,7 +4432,7 @@
         <v>40778.851435954799</v>
       </c>
     </row>
-    <row r="365" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="365" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A365" s="1">
         <v>45413</v>
       </c>
@@ -4443,7 +4443,7 @@
         <v>37842.002628304697</v>
       </c>
     </row>
-    <row r="366" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="366" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A366" s="1">
         <v>45444</v>
       </c>
@@ -4454,7 +4454,7 @@
         <v>33380.999493744603</v>
       </c>
     </row>
-    <row r="367" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="367" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A367" s="1">
         <v>45474</v>
       </c>
@@ -4465,7 +4465,7 @@
         <v>44577.858142612597</v>
       </c>
     </row>
-    <row r="368" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="368" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A368" s="1">
         <v>45505</v>
       </c>
@@ -4476,7 +4476,7 @@
         <v>44325.831029690598</v>
       </c>
     </row>
-    <row r="369" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="369" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A369" s="1">
         <v>45536</v>
       </c>
@@ -4487,7 +4487,7 @@
         <v>43840.785857267998</v>
       </c>
     </row>
-    <row r="370" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="370" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A370" s="1">
         <v>45566</v>
       </c>
@@ -4498,7 +4498,7 @@
         <v>45461.434063650202</v>
       </c>
     </row>
-    <row r="371" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="371" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A371" s="1">
         <v>45597</v>
       </c>
@@ -4509,7 +4509,7 @@
         <v>48044.604332723698</v>
       </c>
     </row>
-    <row r="372" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="372" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A372" s="1">
         <v>45627</v>
       </c>
@@ -4520,7 +4520,7 @@
         <v>46510.342809666698</v>
       </c>
     </row>
-    <row r="373" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="373" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A373" s="1">
         <v>45658</v>
       </c>
@@ -4531,7 +4531,7 @@
         <v>47056.233345127999</v>
       </c>
     </row>
-    <row r="374" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="374" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A374" s="1">
         <v>45689</v>
       </c>
@@ -4542,7 +4542,7 @@
         <v>46750.418887440297</v>
       </c>
     </row>
-    <row r="375" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="375" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A375" s="1">
         <v>45717</v>
       </c>
@@ -4553,7 +4553,7 @@
         <v>37992.202397283603</v>
       </c>
     </row>
-    <row r="376" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="376" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A376" s="1">
         <v>45748</v>
       </c>
@@ -4564,7 +4564,7 @@
         <v>43375.247072162201</v>
       </c>
     </row>
-    <row r="377" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="377" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A377" s="1">
         <v>45778</v>
       </c>
@@ -4575,7 +4575,7 @@
         <v>49106.994792613797</v>
       </c>
     </row>
-    <row r="378" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="378" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A378" s="1">
         <v>45809</v>
       </c>
@@ -4586,7 +4586,7 @@
         <v>42897.329152975399</v>
       </c>
     </row>
-    <row r="379" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="379" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A379" s="1">
         <v>45839</v>
       </c>
@@ -4597,7 +4597,7 @@
         <v>36983.991052674603</v>
       </c>
     </row>
-    <row r="380" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="380" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A380" s="1">
         <v>45870</v>
       </c>
@@ -4608,7 +4608,7 @@
         <v>38426.808349861698</v>
       </c>
     </row>
-    <row r="381" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="381" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A381" s="1">
         <v>45901</v>
       </c>
@@ -4619,7 +4619,7 @@
         <v>39667.366788627398</v>
       </c>
     </row>
-    <row r="382" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="382" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A382" s="1">
         <v>45931</v>
       </c>
@@ -4630,7 +4630,7 @@
         <v>40153.568639117097</v>
       </c>
     </row>
-    <row r="383" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="383" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A383" s="1">
         <v>45962</v>
       </c>
@@ -4641,7 +4641,7 @@
         <v>33970.318844048801</v>
       </c>
     </row>
-    <row r="384" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="384" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A384" s="1">
         <v>45992</v>
       </c>
@@ -4652,7 +4652,7 @@
         <v>33683.521040143198</v>
       </c>
     </row>
-    <row r="385" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="385" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A385" s="1">
         <v>46023</v>
       </c>
@@ -4663,7 +4663,7 @@
         <v>38873.237576069601</v>
       </c>
     </row>
-    <row r="386" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="386" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A386" s="1">
         <v>46054</v>
       </c>
@@ -4674,7 +4674,7 @@
         <v>34234.939050494497</v>
       </c>
     </row>
-    <row r="387" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="387" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A387" s="1">
         <v>46082</v>
       </c>
@@ -4685,7 +4685,7 @@
         <v>36869.134555199802</v>
       </c>
     </row>
-    <row r="388" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="388" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A388" s="1">
         <v>46113</v>
       </c>

</xml_diff>